<commit_message>
Complete all test cases and bug reports for Classroom and Student modules
</commit_message>
<xml_diff>
--- a/Yoedu_Management_Bug_Test.xlsx
+++ b/Yoedu_Management_Bug_Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automate test\Test case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E9EA67-5A1A-4D06-87EC-2F0504B1EF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DA403F4-D8D4-4644-8098-544B4DDBFB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="12180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="12180" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bugs_Phòng_Học" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
   <si>
     <t>Bug</t>
   </si>
@@ -56,6 +56,102 @@
   </si>
   <si>
     <t>Evidence</t>
+  </si>
+  <si>
+    <t>rooms</t>
+  </si>
+  <si>
+    <t>Broken image icon displayed in the "Hình ảnh" section on the Room Details page.</t>
+  </si>
+  <si>
+    <t>Chrome (Latest), Windows</t>
+  </si>
+  <si>
+    <t>1. Go to Classroom list.
+2. Click on the hyperlink of Room Code "PHONG_AUTO_2801".
+3. Scroll down to the "Hình ảnh" section.</t>
+  </si>
+  <si>
+    <t>The image fails to load, showing a broken image icon and the alt text "Ảnh đã chọn".</t>
+  </si>
+  <si>
+    <t>The actual image of the classroom should be displayed. If no image was uploaded, it should show a default placeholder or be hidden.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>evidence/bug003_broken_image.jpg</t>
+  </si>
+  <si>
+    <t>System allows the creation of multiple classrooms with identical Room Codes (Mã).</t>
+  </si>
+  <si>
+    <t>1. Click the + (Add New) button on the Rooms list page.
+2. Enter a Room Code that already exists in the system (e.g., PHONG_AUTO_DUP_001).
+3. Fill in other required fields (Name, etc.).
+4. Click Save (Lưu).</t>
+  </si>
+  <si>
+    <t>The system successfully creates the new room. The data grid displays multiple rooms with the exact same Code.</t>
+  </si>
+  <si>
+    <t>The system must block the creation process and display a validation error message: "Mã phòng học đã tồn tại" (Room code already exists).</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>evidence/bug001_broken_image.jpg</t>
+  </si>
+  <si>
+    <t>The "Mã*" (Room Code) field is editable on the Edit Room page.</t>
+  </si>
+  <si>
+    <t>1. Go to the Rooms list page.
+2. Click the ... action menu on any room and select "Sửa" (Edit).
+3. Click on the "Mã*" input field.</t>
+  </si>
+  <si>
+    <t>The "Mã*" field is fully editable. Users can delete or change the unique room code.</t>
+  </si>
+  <si>
+    <t>The "Mã*" field should be disabled (read-only) in the Edit mode to prevent breaking data integrity and relationships in the database.</t>
+  </si>
+  <si>
+    <t>evidence/bug002_broken_image.jpg</t>
+  </si>
+  <si>
+    <t>Broken image icon displayed in the "Hình ảnh" section on the Edit Room page.</t>
+  </si>
+  <si>
+    <t>1. Go to Edit page of a room (e.g., PH1020).2. Scroll down to the image upload section.</t>
+  </si>
+  <si>
+    <t>A broken image icon with the alt text "Ảnh đã chọn" is displayed below the upload area.</t>
+  </si>
+  <si>
+    <t>It should display the currently saved image of the room. If no image exists, it should be blank or show a proper default placeholder.</t>
+  </si>
+  <si>
+    <t>The "Tải lại trang" (Refresh) button clears all active search criteria and filters instead of just reloading data.</t>
+  </si>
+  <si>
+    <t>studets</t>
+  </si>
+  <si>
+    <t>1. Go to the Students list page.
+2. Enter a keyword in the Search box or apply a filter via "TÌM KIẾM NÂNG CAO".
+3. Click the Refresh (circular arrows) icon.</t>
+  </si>
+  <si>
+    <t>All search inputs and filters are completely cleared, and the table resets to show all records.</t>
+  </si>
+  <si>
+    <t>The Refresh button should only pull the latest data from the server matching the currently applied search criteria and filters. It should NOT wipe out the user's input.</t>
+  </si>
+  <si>
+    <t>Low</t>
   </si>
 </sst>
 </file>
@@ -79,10 +175,36 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -91,8 +213,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -373,39 +508,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="1" max="1" width="3.76953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.04296875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="22.31640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.58984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="92.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="114.2265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.7265625" style="2"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.75">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="206.5" x14ac:dyDescent="0.75">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="118" x14ac:dyDescent="0.75">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="147.5" x14ac:dyDescent="0.75">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="73.75" x14ac:dyDescent="0.75">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -415,17 +685,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E607801C-F1E3-4ED8-9F7F-C342183F3999}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="3.76953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="87.953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.31640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.58984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.31640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.6796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="75.76953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="135.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.2265625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.953125" bestFit="1" customWidth="1"/>
   </cols>
@@ -462,6 +732,35 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2" spans="1:10" ht="147.5" x14ac:dyDescent="0.75">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>